<commit_message>
tidy the scripts, line up the three levels' tables, and stop the scatter calling discordant sets concordant
</commit_message>
<xml_diff>
--- a/04_Network/04_test_modules/c_data/04_test_modules.xlsx
+++ b/04_Network/04_test_modules/c_data/04_test_modules.xlsx
@@ -165,7 +165,7 @@
     <t>04_Network/01_build_modules/c_data/modules.rds</t>
   </si>
   <si>
-    <t>49b98bd219f189de1b47175b0644dd3e</t>
+    <t>d9a37515570be8efb6716b246dda0527</t>
   </si>
   <si>
     <t>design</t>
@@ -192,7 +192,7 @@
     <t>02_Differential_Expression/03_Phenotype/c_data/phenotype.rds</t>
   </si>
   <si>
-    <t>8c3594ce8bc5012ea86d027fc5d641fd</t>
+    <t>7e6093b8f4a130433abe2db512d8b1f0</t>
   </si>
   <si>
     <t>imputed</t>

</xml_diff>